<commit_message>
added initial support for simulation
</commit_message>
<xml_diff>
--- a/src/output/test_output.xlsx
+++ b/src/output/test_output.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>t</t>
   </si>
@@ -116,6 +116,24 @@
   </si>
   <si>
     <t>bus:remoteA:va_c_degree</t>
+  </si>
+  <si>
+    <t>bus:remoteB:vm_a_pu</t>
+  </si>
+  <si>
+    <t>bus:remoteB:va_a_degree</t>
+  </si>
+  <si>
+    <t>bus:remoteB:vm_b_pu</t>
+  </si>
+  <si>
+    <t>bus:remoteB:va_b_degree</t>
+  </si>
+  <si>
+    <t>bus:remoteB:vm_c_pu</t>
+  </si>
+  <si>
+    <t>bus:remoteB:va_c_degree</t>
   </si>
 </sst>
 </file>
@@ -473,10 +491,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI22"/>
+  <dimension ref="A1:AO22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:35">
+    <row r="1" spans="1:41">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,8 +597,26 @@
       <c r="AI1" s="1" t="s">
         <v>33</v>
       </c>
+      <c r="AJ1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="2" spans="1:35">
+    <row r="2" spans="1:41">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -686,8 +722,26 @@
       <c r="AI2">
         <v>118.3058949670522</v>
       </c>
+      <c r="AJ2">
+        <v>0.9829257148501604</v>
+      </c>
+      <c r="AK2">
+        <v>-1.600287068058186</v>
+      </c>
+      <c r="AL2">
+        <v>0.9829257148501601</v>
+      </c>
+      <c r="AM2">
+        <v>-121.6002870680582</v>
+      </c>
+      <c r="AN2">
+        <v>0.9829257148501603</v>
+      </c>
+      <c r="AO2">
+        <v>118.3997129319418</v>
+      </c>
     </row>
-    <row r="3" spans="1:35">
+    <row r="3" spans="1:41">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -793,8 +847,26 @@
       <c r="AI3">
         <v>118.2833161815479</v>
       </c>
+      <c r="AJ3">
+        <v>0.9826903505787675</v>
+      </c>
+      <c r="AK3">
+        <v>-1.621590223844264</v>
+      </c>
+      <c r="AL3">
+        <v>0.9826903505787675</v>
+      </c>
+      <c r="AM3">
+        <v>-121.6215902238443</v>
+      </c>
+      <c r="AN3">
+        <v>0.9826903505787674</v>
+      </c>
+      <c r="AO3">
+        <v>118.3784097761557</v>
+      </c>
     </row>
-    <row r="4" spans="1:35">
+    <row r="4" spans="1:41">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -900,8 +972,26 @@
       <c r="AI4">
         <v>118.2607406412221</v>
       </c>
+      <c r="AJ4">
+        <v>0.9824548803524933</v>
+      </c>
+      <c r="AK4">
+        <v>-1.642889685515492</v>
+      </c>
+      <c r="AL4">
+        <v>0.9824548803524933</v>
+      </c>
+      <c r="AM4">
+        <v>-121.6428896855155</v>
+      </c>
+      <c r="AN4">
+        <v>0.9824548803524932</v>
+      </c>
+      <c r="AO4">
+        <v>118.3571103144845</v>
+      </c>
     </row>
-    <row r="5" spans="1:35">
+    <row r="5" spans="1:41">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -1007,8 +1097,26 @@
       <c r="AI5">
         <v>118.2381838227807</v>
       </c>
+      <c r="AJ5">
+        <v>0.9822194658485601</v>
+      </c>
+      <c r="AK5">
+        <v>-1.664170851219349</v>
+      </c>
+      <c r="AL5">
+        <v>0.9822194658485599</v>
+      </c>
+      <c r="AM5">
+        <v>-121.6641708512194</v>
+      </c>
+      <c r="AN5">
+        <v>0.9822194658485599</v>
+      </c>
+      <c r="AO5">
+        <v>118.3358291487806</v>
+      </c>
     </row>
-    <row r="6" spans="1:35">
+    <row r="6" spans="1:41">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -1114,8 +1222,26 @@
       <c r="AI6">
         <v>118.215661215348</v>
       </c>
+      <c r="AJ6">
+        <v>0.9819842692563671</v>
+      </c>
+      <c r="AK6">
+        <v>-1.68541910912456</v>
+      </c>
+      <c r="AL6">
+        <v>0.9819842692563669</v>
+      </c>
+      <c r="AM6">
+        <v>-121.6854191091246</v>
+      </c>
+      <c r="AN6">
+        <v>0.9819842692563669</v>
+      </c>
+      <c r="AO6">
+        <v>118.3145808908754</v>
+      </c>
     </row>
-    <row r="7" spans="1:35">
+    <row r="7" spans="1:41">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1221,8 +1347,26 @@
       <c r="AI7">
         <v>118.1931883098836</v>
       </c>
+      <c r="AJ7">
+        <v>0.9817494531658117</v>
+      </c>
+      <c r="AK7">
+        <v>-1.706619847408013</v>
+      </c>
+      <c r="AL7">
+        <v>0.9817494531658119</v>
+      </c>
+      <c r="AM7">
+        <v>-121.706619847408</v>
+      </c>
+      <c r="AN7">
+        <v>0.9817494531658119</v>
+      </c>
+      <c r="AO7">
+        <v>118.293380152592</v>
+      </c>
     </row>
-    <row r="8" spans="1:35">
+    <row r="8" spans="1:41">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -1328,8 +1472,26 @@
       <c r="AI8">
         <v>118.1707805885267</v>
       </c>
+      <c r="AJ8">
+        <v>0.9815151804538269</v>
+      </c>
+      <c r="AK8">
+        <v>-1.727758464304553</v>
+      </c>
+      <c r="AL8">
+        <v>0.981515180453827</v>
+      </c>
+      <c r="AM8">
+        <v>-121.7277584643045</v>
+      </c>
+      <c r="AN8">
+        <v>0.981515180453827</v>
+      </c>
+      <c r="AO8">
+        <v>118.2722415356954</v>
+      </c>
     </row>
-    <row r="9" spans="1:35">
+    <row r="9" spans="1:41">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1435,8 +1597,26 @@
       <c r="AI9">
         <v>118.1484535138768</v>
       </c>
+      <c r="AJ9">
+        <v>0.9812816141691766</v>
+      </c>
+      <c r="AK9">
+        <v>-1.74882037821283</v>
+      </c>
+      <c r="AL9">
+        <v>0.9812816141691767</v>
+      </c>
+      <c r="AM9">
+        <v>-121.7488203782128</v>
+      </c>
+      <c r="AN9">
+        <v>0.9812816141691767</v>
+      </c>
+      <c r="AO9">
+        <v>118.2511796217871</v>
+      </c>
     </row>
-    <row r="10" spans="1:35">
+    <row r="10" spans="1:41">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -1542,8 +1722,26 @@
       <c r="AI10">
         <v>118.126222518216</v>
       </c>
+      <c r="AJ10">
+        <v>0.9810489174156352</v>
+      </c>
+      <c r="AK10">
+        <v>-1.769791037850871</v>
+      </c>
+      <c r="AL10">
+        <v>0.9810489174156349</v>
+      </c>
+      <c r="AM10">
+        <v>-121.7697910378509</v>
+      </c>
+      <c r="AN10">
+        <v>0.981048917415635</v>
+      </c>
+      <c r="AO10">
+        <v>118.2302089621491</v>
+      </c>
     </row>
-    <row r="11" spans="1:35">
+    <row r="11" spans="1:41">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -1649,8 +1847,26 @@
       <c r="AI11">
         <v>118.1041029926803</v>
       </c>
+      <c r="AJ11">
+        <v>0.9808172532335663</v>
+      </c>
+      <c r="AK11">
+        <v>-1.790655932454542</v>
+      </c>
+      <c r="AL11">
+        <v>0.9808172532335663</v>
+      </c>
+      <c r="AM11">
+        <v>-121.7906559324545</v>
+      </c>
+      <c r="AN11">
+        <v>0.9808172532335662</v>
+      </c>
+      <c r="AO11">
+        <v>118.2093440675454</v>
+      </c>
     </row>
-    <row r="12" spans="1:35">
+    <row r="12" spans="1:41">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -1756,8 +1972,26 @@
       <c r="AI12">
         <v>116.7516369243639</v>
       </c>
+      <c r="AJ12">
+        <v>0.9621563369337319</v>
+      </c>
+      <c r="AK12">
+        <v>-3.815969084416833</v>
+      </c>
+      <c r="AL12">
+        <v>0.9621563369337318</v>
+      </c>
+      <c r="AM12">
+        <v>-123.8159690844168</v>
+      </c>
+      <c r="AN12">
+        <v>0.9621563369337319</v>
+      </c>
+      <c r="AO12">
+        <v>116.1840309155832</v>
+      </c>
     </row>
-    <row r="13" spans="1:35">
+    <row r="13" spans="1:41">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -1810,7 +2044,7 @@
         <v>4.336808689942018E-19</v>
       </c>
     </row>
-    <row r="14" spans="1:35">
+    <row r="14" spans="1:41">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -1863,7 +2097,7 @@
         <v>4.336808689942018E-19</v>
       </c>
     </row>
-    <row r="15" spans="1:35">
+    <row r="15" spans="1:41">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -1916,7 +2150,7 @@
         <v>4.336808689942018E-19</v>
       </c>
     </row>
-    <row r="16" spans="1:35">
+    <row r="16" spans="1:41">
       <c r="A16" s="1">
         <v>14</v>
       </c>

</xml_diff>